<commit_message>
chore: delete E2 (duplicate of E1) and update D1 to show empty data
- E2 removed: same scenario as E1 (BM + has pref sols), now only E1 remains
- D1 updated: BM no pref with sahayog_branch shows empty/0 rows data
</commit_message>
<xml_diff>
--- a/role_table_test_cases.xlsx
+++ b/role_table_test_cases.xlsx
@@ -628,7 +628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="17" min="1" max="1"/>
@@ -1626,69 +1626,78 @@
       </c>
       <c r="E14" s="25" t="inlineStr">
         <is>
-          <t>TRUE
-(fallback)</t>
+          <t>TRUE but empty</t>
         </is>
       </c>
       <c r="F14" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [1000] </t>
+          <t xml:space="preserve"> [1000] → 0 rows</t>
         </is>
       </c>
       <c r="G14" s="26" t="inlineStr">
         <is>
-          <t>Only 1000</t>
+          <t>Empty
+0 rows</t>
         </is>
       </c>
       <c r="H14" s="26" t="inlineStr">
         <is>
-          <t>Only 1000</t>
+          <t>Empty
+0 rows</t>
         </is>
       </c>
       <c r="I14" s="26" t="inlineStr">
         <is>
-          <t>Only 1000</t>
+          <t>Empty
+0 rows</t>
         </is>
       </c>
       <c r="J14" s="26" t="inlineStr">
         <is>
-          <t>Only 1000</t>
+          <t>Empty
+0 rows</t>
         </is>
       </c>
       <c r="K14" s="26" t="inlineStr">
         <is>
-          <t>Only 1000</t>
+          <t>Empty
+0 rows</t>
         </is>
       </c>
       <c r="L14" s="26" t="inlineStr">
         <is>
-          <t>Only 1000 staff</t>
+          <t>Empty
+0 rows</t>
         </is>
       </c>
       <c r="M14" s="26" t="inlineStr">
         <is>
-          <t>Only 1000</t>
+          <t>Empty
+0 rows</t>
         </is>
       </c>
       <c r="N14" s="26" t="inlineStr">
         <is>
-          <t>Only 1000</t>
+          <t>Empty
+0 rows</t>
         </is>
       </c>
       <c r="O14" s="26" t="inlineStr">
         <is>
-          <t>Only 1000</t>
+          <t>Empty
+0 rows</t>
         </is>
       </c>
       <c r="P14" s="26" t="inlineStr">
         <is>
-          <t>Only 1000</t>
+          <t>Empty
+0 rows</t>
         </is>
       </c>
       <c r="Q14" s="25" t="inlineStr">
         <is>
-          <t>YES
-single SOL</t>
+          <t>YES but
+empty data</t>
         </is>
       </c>
     </row>
@@ -1976,7 +1985,7 @@
     <row r="18" ht="33.75" customHeight="1" s="18">
       <c r="A18" s="23" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="B18" s="23" t="inlineStr">
@@ -1987,8 +1996,7 @@
       </c>
       <c r="C18" s="23" t="inlineStr">
         <is>
-          <t>Sols [1001,1002]
-(2 SOLs) + Employee 1000</t>
+          <t>Zones [ZONE-1] + Employee 1000</t>
         </is>
       </c>
       <c r="D18" s="23" t="inlineStr">
@@ -2002,252 +2010,163 @@
         </is>
       </c>
       <c r="F18" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> [1001,1002]
-(pref wins, Emp ignored)</t>
-        </is>
-      </c>
-      <c r="G18" s="26" t="inlineStr">
-        <is>
-          <t>Only 1001,1002</t>
-        </is>
-      </c>
-      <c r="H18" s="26" t="inlineStr">
-        <is>
-          <t>Only 1001,1002</t>
-        </is>
-      </c>
-      <c r="I18" s="26" t="inlineStr">
-        <is>
-          <t>Only 1001,1002</t>
-        </is>
-      </c>
-      <c r="J18" s="26" t="inlineStr">
-        <is>
-          <t>Only 1001,1002</t>
-        </is>
-      </c>
-      <c r="K18" s="26" t="inlineStr">
-        <is>
-          <t>Only 1001,1002</t>
-        </is>
-      </c>
-      <c r="L18" s="26" t="inlineStr">
-        <is>
-          <t>Only 1001,1002 staff</t>
-        </is>
-      </c>
-      <c r="M18" s="26" t="inlineStr">
-        <is>
-          <t>Only 1001,1002</t>
-        </is>
-      </c>
-      <c r="N18" s="26" t="inlineStr">
-        <is>
-          <t>Only 1001,1002</t>
-        </is>
-      </c>
-      <c r="O18" s="26" t="inlineStr">
-        <is>
-          <t>Only 1001,1002</t>
-        </is>
-      </c>
-      <c r="P18" s="26" t="inlineStr">
-        <is>
-          <t>Only 1001,1002</t>
-        </is>
-      </c>
-      <c r="Q18" s="26" t="inlineStr">
-        <is>
-          <t>YES
-pref SOLs</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="33.75" customHeight="1" s="18">
-      <c r="A19" s="23" t="inlineStr">
-        <is>
-          <t>E3</t>
-        </is>
-      </c>
-      <c r="B19" s="23" t="inlineStr">
-        <is>
-          <t>User is BM
-+ has Pref</t>
-        </is>
-      </c>
-      <c r="C19" s="23" t="inlineStr">
-        <is>
-          <t>Zones [ZONE-1] + Employee 1000</t>
-        </is>
-      </c>
-      <c r="D19" s="23" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="E19" s="25" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="F19" s="23" t="inlineStr">
         <is>
           <t>ZONE-1
 (Employee ignored
 when pref has zones)</t>
         </is>
       </c>
-      <c r="G19" s="26" t="inlineStr">
+      <c r="G18" s="26" t="inlineStr">
         <is>
           <t>Only ZONE-1</t>
         </is>
       </c>
-      <c r="H19" s="26" t="inlineStr">
+      <c r="H18" s="26" t="inlineStr">
         <is>
           <t>Only ZONE-1</t>
         </is>
       </c>
-      <c r="I19" s="26" t="inlineStr">
+      <c r="I18" s="26" t="inlineStr">
         <is>
           <t>Only ZONE-1</t>
         </is>
       </c>
-      <c r="J19" s="26" t="inlineStr">
+      <c r="J18" s="26" t="inlineStr">
         <is>
           <t>Only ZONE-1</t>
         </is>
       </c>
-      <c r="K19" s="26" t="inlineStr">
+      <c r="K18" s="26" t="inlineStr">
         <is>
           <t>Only ZONE-1</t>
         </is>
       </c>
-      <c r="L19" s="26" t="inlineStr">
+      <c r="L18" s="26" t="inlineStr">
         <is>
           <t>Only ZONE-1 staff</t>
         </is>
       </c>
-      <c r="M19" s="26" t="inlineStr">
+      <c r="M18" s="26" t="inlineStr">
         <is>
           <t>Only ZONE-1</t>
         </is>
       </c>
-      <c r="N19" s="26" t="inlineStr">
+      <c r="N18" s="26" t="inlineStr">
         <is>
           <t>Only ZONE-1</t>
         </is>
       </c>
-      <c r="O19" s="26" t="inlineStr">
+      <c r="O18" s="26" t="inlineStr">
         <is>
           <t>Only ZONE-1</t>
         </is>
       </c>
-      <c r="P19" s="26" t="inlineStr">
+      <c r="P18" s="26" t="inlineStr">
         <is>
           <t>Only ZONE-1</t>
         </is>
       </c>
-      <c r="Q19" s="26" t="inlineStr">
+      <c r="Q18" s="26" t="inlineStr">
         <is>
           <t>YES
 zone filter</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="33.75" customHeight="1" s="18">
-      <c r="A20" s="23" t="inlineStr">
+    <row r="19" ht="33.75" customHeight="1" s="18">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>E4</t>
         </is>
       </c>
-      <c r="B20" s="23" t="inlineStr">
+      <c r="B19" s="23" t="inlineStr">
         <is>
           <t>User is BM
 + has Pref</t>
         </is>
       </c>
-      <c r="C20" s="23" t="inlineStr">
+      <c r="C19" s="23" t="inlineStr">
         <is>
           <t>Sols [] Zones [] Regions []
 all_regions FALSE
 (Employee 1000)</t>
         </is>
       </c>
-      <c r="D20" s="23" t="inlineStr">
+      <c r="D19" s="23" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="E20" s="25" t="inlineStr">
+      <c r="E19" s="25" t="inlineStr">
         <is>
           <t>TRUE
 (fallback to
 Employee)</t>
         </is>
       </c>
-      <c r="F20" s="23" t="inlineStr">
+      <c r="F19" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve"> [1000] </t>
         </is>
       </c>
-      <c r="G20" s="26" t="inlineStr">
+      <c r="G19" s="26" t="inlineStr">
         <is>
           <t>Only 1000</t>
         </is>
       </c>
-      <c r="H20" s="26" t="inlineStr">
+      <c r="H19" s="26" t="inlineStr">
         <is>
           <t>Only 1000</t>
         </is>
       </c>
-      <c r="I20" s="26" t="inlineStr">
+      <c r="I19" s="26" t="inlineStr">
         <is>
           <t>Only 1000</t>
         </is>
       </c>
-      <c r="J20" s="26" t="inlineStr">
+      <c r="J19" s="26" t="inlineStr">
         <is>
           <t>Only 1000</t>
         </is>
       </c>
-      <c r="K20" s="26" t="inlineStr">
+      <c r="K19" s="26" t="inlineStr">
         <is>
           <t>Only 1000</t>
         </is>
       </c>
-      <c r="L20" s="26" t="inlineStr">
+      <c r="L19" s="26" t="inlineStr">
         <is>
           <t>Only 1000 staff</t>
         </is>
       </c>
-      <c r="M20" s="26" t="inlineStr">
+      <c r="M19" s="26" t="inlineStr">
         <is>
           <t>Only 1000</t>
         </is>
       </c>
-      <c r="N20" s="26" t="inlineStr">
+      <c r="N19" s="26" t="inlineStr">
         <is>
           <t>Only 1000</t>
         </is>
       </c>
-      <c r="O20" s="26" t="inlineStr">
+      <c r="O19" s="26" t="inlineStr">
         <is>
           <t>Only 1000</t>
         </is>
       </c>
-      <c r="P20" s="26" t="inlineStr">
+      <c r="P19" s="26" t="inlineStr">
         <is>
           <t>Only 1000</t>
         </is>
       </c>
-      <c r="Q20" s="26" t="inlineStr">
+      <c r="Q19" s="26" t="inlineStr">
         <is>
           <t>YES
 fallback</t>
         </is>
       </c>
     </row>
+    <row r="20" ht="33.75" customHeight="1" s="18"/>
     <row r="1048576" ht="12.8" customHeight="1" s="18"/>
   </sheetData>
   <autoFilter ref="A4:Q20"/>

</xml_diff>